<commit_message>
added Weather Station settings
</commit_message>
<xml_diff>
--- a/Antonio-Feed/__FeedPartsInventory.xlsx
+++ b/Antonio-Feed/__FeedPartsInventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pollak/Documents/GitHub/Front-Page/Antonio-Feed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD42A30A-8723-8C4B-BDAF-BB195EB8564D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FBBDE6F-6D51-AB40-8D23-E28C724EAF1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-93320" yWindow="7020" windowWidth="34200" windowHeight="19940" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-100000" yWindow="600" windowWidth="34200" windowHeight="19940" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts At ATA" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
   <definedNames>
     <definedName name="xx_1" localSheetId="0">'Parts At ATA'!$A$2:$G$44</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1266" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="451">
   <si>
     <t>Antenna Inventory</t>
   </si>
@@ -1342,6 +1342,60 @@
   </si>
   <si>
     <t xml:space="preserve">Vds=1.20V </t>
+  </si>
+  <si>
+    <t>5C4-027</t>
+  </si>
+  <si>
+    <t>5C4-028</t>
+  </si>
+  <si>
+    <t>5C4-029</t>
+  </si>
+  <si>
+    <t>5C4-030</t>
+  </si>
+  <si>
+    <t>5C4-031</t>
+  </si>
+  <si>
+    <t>5C4-032</t>
+  </si>
+  <si>
+    <t>5C4-033</t>
+  </si>
+  <si>
+    <t>5C4-034</t>
+  </si>
+  <si>
+    <t>5C4-035</t>
+  </si>
+  <si>
+    <t>5C4-036</t>
+  </si>
+  <si>
+    <t>5C4-037</t>
+  </si>
+  <si>
+    <t>5C4-038</t>
+  </si>
+  <si>
+    <t>5C4-039</t>
+  </si>
+  <si>
+    <t>5C4-040</t>
+  </si>
+  <si>
+    <t>5C4-041</t>
+  </si>
+  <si>
+    <t>5C4-042</t>
+  </si>
+  <si>
+    <t>5C4-043</t>
+  </si>
+  <si>
+    <t>5C4-044</t>
   </si>
 </sst>
 </file>
@@ -1458,7 +1512,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1591,8 +1645,14 @@
         <bgColor rgb="FFFF9900"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="24">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -1879,12 +1939,60 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="131">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1996,7 +2104,6 @@
     <xf numFmtId="0" fontId="4" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2084,6 +2191,10 @@
     <xf numFmtId="0" fontId="4" fillId="20" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="21" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="22" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2123,10 +2234,22 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2365,25 +2488,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="108" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="109"/>
-      <c r="I1" s="110"/>
-      <c r="J1" s="110"/>
-      <c r="K1" s="109"/>
-      <c r="L1" s="110"/>
-      <c r="M1" s="110"/>
-      <c r="N1" s="110"/>
-      <c r="O1" s="110"/>
-      <c r="P1" s="110"/>
-      <c r="Q1" s="110"/>
+      <c r="B1" s="109"/>
+      <c r="C1" s="109"/>
+      <c r="D1" s="109"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="109"/>
+      <c r="G1" s="109"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="111"/>
+      <c r="O1" s="111"/>
+      <c r="P1" s="111"/>
+      <c r="Q1" s="111"/>
     </row>
     <row r="2" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -3695,28 +3818,28 @@
       <c r="A58" s="3"/>
     </row>
     <row r="59" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="111"/>
-      <c r="B59" s="106"/>
-      <c r="C59" s="106"/>
+      <c r="A59" s="112"/>
+      <c r="B59" s="107"/>
+      <c r="C59" s="107"/>
     </row>
     <row r="60" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="7"/>
     </row>
     <row r="61" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="105"/>
-      <c r="B61" s="106"/>
-      <c r="C61" s="105"/>
-      <c r="D61" s="106"/>
-      <c r="E61" s="106"/>
-      <c r="F61" s="106"/>
+      <c r="A61" s="106"/>
+      <c r="B61" s="107"/>
+      <c r="C61" s="106"/>
+      <c r="D61" s="107"/>
+      <c r="E61" s="107"/>
+      <c r="F61" s="107"/>
     </row>
     <row r="62" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="105"/>
-      <c r="B62" s="106"/>
-      <c r="C62" s="105"/>
-      <c r="D62" s="106"/>
-      <c r="E62" s="106"/>
-      <c r="F62" s="106"/>
+      <c r="A62" s="106"/>
+      <c r="B62" s="107"/>
+      <c r="C62" s="106"/>
+      <c r="D62" s="107"/>
+      <c r="E62" s="107"/>
+      <c r="F62" s="107"/>
     </row>
     <row r="63" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="64" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4681,7 +4804,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -4693,20 +4816,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="113" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="114" t="s">
+      <c r="B1" s="114"/>
+      <c r="C1" s="115" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="115"/>
-      <c r="E1" s="115"/>
-      <c r="F1" s="115"/>
-      <c r="G1" s="115"/>
-      <c r="H1" s="115"/>
-      <c r="I1" s="115"/>
-      <c r="J1" s="115"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
+      <c r="H1" s="116"/>
+      <c r="I1" s="116"/>
+      <c r="J1" s="116"/>
       <c r="K1" s="9"/>
       <c r="L1" s="9"/>
     </row>
@@ -4786,7 +4909,7 @@
         <v>317</v>
       </c>
       <c r="L3" s="38"/>
-      <c r="M3" s="99"/>
+      <c r="M3" s="98"/>
     </row>
     <row r="4" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="str">
@@ -4824,7 +4947,7 @@
         <v>311</v>
       </c>
       <c r="L4" s="12"/>
-      <c r="M4" s="99"/>
+      <c r="M4" s="98"/>
     </row>
     <row r="5" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="str">
@@ -4862,14 +4985,14 @@
         <v>318</v>
       </c>
       <c r="L5" s="38"/>
-      <c r="M5" s="99"/>
+      <c r="M5" s="98"/>
     </row>
     <row r="6" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="str">
         <f>HYPERLINK("https://drive.google.com/drive/folders/1WeIiiMAp6TYYdsybsr5MvXeiX_cVX9j0","5C4-004")</f>
         <v>5C4-004</v>
       </c>
-      <c r="B6" s="104" t="s">
+      <c r="B6" s="103" t="s">
         <v>126</v>
       </c>
       <c r="C6" s="15" t="s">
@@ -4902,7 +5025,7 @@
       <c r="L6" s="38" t="s">
         <v>282</v>
       </c>
-      <c r="M6" s="99"/>
+      <c r="M6" s="98"/>
     </row>
     <row r="7" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="13" t="str">
@@ -4942,7 +5065,7 @@
       <c r="L7" s="38" t="s">
         <v>320</v>
       </c>
-      <c r="M7" s="99"/>
+      <c r="M7" s="98"/>
     </row>
     <row r="8" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="13" t="str">
@@ -4982,7 +5105,7 @@
       <c r="L8" s="38" t="s">
         <v>320</v>
       </c>
-      <c r="M8" s="99"/>
+      <c r="M8" s="98"/>
     </row>
     <row r="9" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="16" t="s">
@@ -5019,7 +5142,7 @@
         <v>290</v>
       </c>
       <c r="L9" s="38"/>
-      <c r="M9" s="99"/>
+      <c r="M9" s="98"/>
     </row>
     <row r="10" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="13" t="str">
@@ -5059,7 +5182,7 @@
       <c r="L10" s="38" t="s">
         <v>282</v>
       </c>
-      <c r="M10" s="99"/>
+      <c r="M10" s="98"/>
     </row>
     <row r="11" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="13" t="str">
@@ -5097,7 +5220,7 @@
         <v>404</v>
       </c>
       <c r="L11" s="38"/>
-      <c r="M11" s="99"/>
+      <c r="M11" s="98"/>
     </row>
     <row r="12" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="13" t="str">
@@ -5135,7 +5258,7 @@
         <v>310</v>
       </c>
       <c r="L12" s="38"/>
-      <c r="M12" s="99"/>
+      <c r="M12" s="98"/>
     </row>
     <row r="13" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="13" t="str">
@@ -5175,7 +5298,7 @@
       <c r="L13" s="38" t="s">
         <v>282</v>
       </c>
-      <c r="M13" s="99"/>
+      <c r="M13" s="98"/>
     </row>
     <row r="14" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="13" t="str">
@@ -5215,7 +5338,7 @@
       <c r="L14" s="38" t="s">
         <v>320</v>
       </c>
-      <c r="M14" s="99"/>
+      <c r="M14" s="98"/>
     </row>
     <row r="15" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="13" t="str">
@@ -5255,7 +5378,7 @@
       <c r="L15" s="38" t="s">
         <v>320</v>
       </c>
-      <c r="M15" s="99"/>
+      <c r="M15" s="98"/>
     </row>
     <row r="16" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="13" t="str">
@@ -5295,7 +5418,7 @@
       <c r="L16" s="38" t="s">
         <v>283</v>
       </c>
-      <c r="M16" s="99"/>
+      <c r="M16" s="98"/>
     </row>
     <row r="17" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="13" t="str">
@@ -5333,13 +5456,13 @@
         <v>314</v>
       </c>
       <c r="L17" s="38"/>
-      <c r="M17" s="99"/>
+      <c r="M17" s="98"/>
     </row>
     <row r="18" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="B18" s="103" t="s">
+      <c r="B18" s="102" t="s">
         <v>237</v>
       </c>
       <c r="C18" s="15" t="s">
@@ -5370,7 +5493,7 @@
         <v>304</v>
       </c>
       <c r="L18" s="38"/>
-      <c r="M18" s="99"/>
+      <c r="M18" s="98"/>
     </row>
     <row r="19" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="13" t="str">
@@ -5408,7 +5531,7 @@
         <v>309</v>
       </c>
       <c r="L19" s="38"/>
-      <c r="M19" s="99"/>
+      <c r="M19" s="98"/>
     </row>
     <row r="20" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="16" t="s">
@@ -5447,7 +5570,7 @@
       <c r="L20" s="38" t="s">
         <v>320</v>
       </c>
-      <c r="M20" s="99"/>
+      <c r="M20" s="98"/>
     </row>
     <row r="21" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="13" t="str">
@@ -5487,86 +5610,86 @@
       <c r="L21" s="38" t="s">
         <v>320</v>
       </c>
-      <c r="M21" s="99"/>
+      <c r="M21" s="98"/>
     </row>
     <row r="22" spans="1:13" ht="16" x14ac:dyDescent="0.2">
-      <c r="A22" s="77" t="str">
+      <c r="A22" s="76" t="str">
         <f>HYPERLINK("https://drive.google.com/drive/folders/1wMVARUxnYHeiTbbEodCmZFb_vx9FkRVr","5C4-020")</f>
         <v>5C4-020</v>
       </c>
-      <c r="B22" s="102" t="s">
+      <c r="B22" s="101" t="s">
         <v>135</v>
       </c>
-      <c r="C22" s="78" t="s">
-        <v>25</v>
-      </c>
-      <c r="D22" s="79" t="s">
-        <v>25</v>
-      </c>
-      <c r="E22" s="79" t="s">
-        <v>25</v>
-      </c>
-      <c r="F22" s="79" t="s">
-        <v>25</v>
-      </c>
-      <c r="G22" s="80" t="s">
-        <v>25</v>
-      </c>
-      <c r="H22" s="79" t="s">
-        <v>25</v>
-      </c>
-      <c r="I22" s="79" t="s">
-        <v>25</v>
-      </c>
-      <c r="J22" s="79" t="s">
-        <v>25</v>
-      </c>
-      <c r="K22" s="81" t="s">
+      <c r="C22" s="77" t="s">
+        <v>25</v>
+      </c>
+      <c r="D22" s="78" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" s="78" t="s">
+        <v>25</v>
+      </c>
+      <c r="F22" s="78" t="s">
+        <v>25</v>
+      </c>
+      <c r="G22" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="H22" s="78" t="s">
+        <v>25</v>
+      </c>
+      <c r="I22" s="78" t="s">
+        <v>25</v>
+      </c>
+      <c r="J22" s="78" t="s">
+        <v>25</v>
+      </c>
+      <c r="K22" s="80" t="s">
         <v>326</v>
       </c>
-      <c r="L22" s="81" t="s">
+      <c r="L22" s="80" t="s">
         <v>320</v>
       </c>
-      <c r="M22" s="100">
+      <c r="M22" s="99">
         <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="75" t="s">
+      <c r="A23" s="74" t="s">
         <v>327</v>
       </c>
-      <c r="B23" s="87" t="s">
+      <c r="B23" s="86" t="s">
         <v>191</v>
       </c>
-      <c r="C23" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="D23" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="E23" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="F23" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="G23" s="80" t="s">
-        <v>25</v>
-      </c>
-      <c r="H23" s="80" t="s">
-        <v>25</v>
-      </c>
-      <c r="I23" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="J23" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="K23" s="81" t="s">
+      <c r="C23" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="F23" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="G23" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="H23" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="I23" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="J23" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="K23" s="80" t="s">
         <v>408</v>
       </c>
       <c r="L23" s="12"/>
-      <c r="M23" s="101">
+      <c r="M23" s="100">
         <v>21</v>
       </c>
     </row>
@@ -5574,38 +5697,38 @@
       <c r="A24" s="16" t="s">
         <v>328</v>
       </c>
-      <c r="B24" s="87" t="s">
+      <c r="B24" s="86" t="s">
         <v>205</v>
       </c>
-      <c r="C24" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="D24" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="E24" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="F24" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="G24" s="80" t="s">
-        <v>25</v>
-      </c>
-      <c r="H24" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="I24" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="J24" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="K24" s="81" t="s">
+      <c r="C24" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="D24" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="G24" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="H24" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="I24" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="J24" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="K24" s="80" t="s">
         <v>414</v>
       </c>
       <c r="L24" s="38"/>
-      <c r="M24" s="101">
+      <c r="M24" s="100">
         <v>22</v>
       </c>
     </row>
@@ -5613,38 +5736,38 @@
       <c r="A25" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="B25" s="87" t="s">
+      <c r="B25" s="86" t="s">
         <v>200</v>
       </c>
-      <c r="C25" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="D25" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="E25" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="F25" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="G25" s="80" t="s">
-        <v>25</v>
-      </c>
-      <c r="H25" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="I25" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="J25" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="K25" s="81" t="s">
+      <c r="C25" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="F25" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="G25" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="H25" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="I25" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="J25" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="K25" s="80" t="s">
         <v>415</v>
       </c>
       <c r="L25" s="38"/>
-      <c r="M25" s="101">
+      <c r="M25" s="100">
         <v>23</v>
       </c>
     </row>
@@ -5652,38 +5775,38 @@
       <c r="A26" s="16" t="s">
         <v>405</v>
       </c>
-      <c r="B26" s="87" t="s">
+      <c r="B26" s="86" t="s">
         <v>157</v>
       </c>
-      <c r="C26" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="D26" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="E26" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="F26" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="G26" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="H26" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="I26" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="J26" s="76" t="s">
+      <c r="C26" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="D26" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="F26" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="G26" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="H26" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="I26" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="J26" s="75" t="s">
         <v>25</v>
       </c>
       <c r="K26" s="38" t="s">
         <v>419</v>
       </c>
       <c r="L26" s="38"/>
-      <c r="M26" s="101">
+      <c r="M26" s="100">
         <v>24</v>
       </c>
     </row>
@@ -5691,38 +5814,38 @@
       <c r="A27" s="16" t="s">
         <v>406</v>
       </c>
-      <c r="B27" s="87" t="s">
+      <c r="B27" s="86" t="s">
         <v>232</v>
       </c>
-      <c r="C27" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="D27" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="E27" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="F27" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="G27" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="H27" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="I27" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="J27" s="76" t="s">
+      <c r="C27" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="D27" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="F27" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="G27" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="H27" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="I27" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="J27" s="75" t="s">
         <v>25</v>
       </c>
       <c r="K27" s="38" t="s">
         <v>420</v>
       </c>
       <c r="L27" s="38"/>
-      <c r="M27" s="101">
+      <c r="M27" s="100">
         <v>25</v>
       </c>
     </row>
@@ -5730,34 +5853,377 @@
       <c r="A28" s="16" t="s">
         <v>407</v>
       </c>
-      <c r="B28" s="59" t="s">
+      <c r="B28" s="124" t="s">
         <v>417</v>
       </c>
-      <c r="C28" s="61"/>
-      <c r="D28" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="E28" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="F28" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="G28" s="38"/>
-      <c r="H28" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="I28" s="38"/>
-      <c r="J28" s="38"/>
-      <c r="K28" s="38"/>
-      <c r="L28" s="38"/>
-      <c r="M28" s="99"/>
+      <c r="C28" s="125"/>
+      <c r="D28" s="126" t="s">
+        <v>25</v>
+      </c>
+      <c r="E28" s="126" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28" s="126" t="s">
+        <v>25</v>
+      </c>
+      <c r="G28" s="127"/>
+      <c r="H28" s="126" t="s">
+        <v>25</v>
+      </c>
+      <c r="I28" s="127"/>
+      <c r="J28" s="127"/>
+      <c r="K28" s="127"/>
+      <c r="L28" s="127"/>
+      <c r="M28" s="128"/>
+    </row>
+    <row r="29" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="123" t="s">
+        <v>433</v>
+      </c>
+      <c r="B29" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C29" s="54"/>
+      <c r="D29" s="129"/>
+      <c r="E29" s="129"/>
+      <c r="F29" s="129"/>
+      <c r="G29" s="129"/>
+      <c r="H29" s="129"/>
+      <c r="I29" s="129"/>
+      <c r="J29" s="129"/>
+      <c r="K29" s="129"/>
+      <c r="L29" s="129"/>
+      <c r="M29" s="129"/>
+    </row>
+    <row r="30" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="123" t="s">
+        <v>434</v>
+      </c>
+      <c r="B30" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C30" s="54"/>
+      <c r="D30" s="129"/>
+      <c r="E30" s="129"/>
+      <c r="F30" s="129"/>
+      <c r="G30" s="129"/>
+      <c r="H30" s="129"/>
+      <c r="I30" s="129"/>
+      <c r="J30" s="129"/>
+      <c r="K30" s="129"/>
+      <c r="L30" s="129"/>
+      <c r="M30" s="129"/>
+    </row>
+    <row r="31" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="123" t="s">
+        <v>435</v>
+      </c>
+      <c r="B31" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C31" s="54"/>
+      <c r="D31" s="129"/>
+      <c r="E31" s="129"/>
+      <c r="F31" s="129"/>
+      <c r="G31" s="129"/>
+      <c r="H31" s="129"/>
+      <c r="I31" s="129"/>
+      <c r="J31" s="129"/>
+      <c r="K31" s="129"/>
+      <c r="L31" s="129"/>
+      <c r="M31" s="129"/>
+    </row>
+    <row r="32" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="123" t="s">
+        <v>436</v>
+      </c>
+      <c r="B32" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C32" s="54"/>
+      <c r="D32" s="129"/>
+      <c r="E32" s="129"/>
+      <c r="F32" s="129"/>
+      <c r="G32" s="129"/>
+      <c r="H32" s="129"/>
+      <c r="I32" s="129"/>
+      <c r="J32" s="129"/>
+      <c r="K32" s="129"/>
+      <c r="L32" s="129"/>
+      <c r="M32" s="129"/>
+    </row>
+    <row r="33" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="123" t="s">
+        <v>437</v>
+      </c>
+      <c r="B33" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C33" s="54"/>
+      <c r="D33" s="129"/>
+      <c r="E33" s="129"/>
+      <c r="F33" s="129"/>
+      <c r="G33" s="129"/>
+      <c r="H33" s="129"/>
+      <c r="I33" s="129"/>
+      <c r="J33" s="129"/>
+      <c r="K33" s="129"/>
+      <c r="L33" s="129"/>
+      <c r="M33" s="129"/>
+    </row>
+    <row r="34" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="123" t="s">
+        <v>438</v>
+      </c>
+      <c r="B34" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C34" s="54"/>
+      <c r="D34" s="129"/>
+      <c r="E34" s="129"/>
+      <c r="F34" s="129"/>
+      <c r="G34" s="129"/>
+      <c r="H34" s="129"/>
+      <c r="I34" s="129"/>
+      <c r="J34" s="129"/>
+      <c r="K34" s="129"/>
+      <c r="L34" s="129"/>
+      <c r="M34" s="129"/>
+    </row>
+    <row r="35" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="123" t="s">
+        <v>439</v>
+      </c>
+      <c r="B35" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C35" s="54"/>
+      <c r="D35" s="129"/>
+      <c r="E35" s="129"/>
+      <c r="F35" s="129"/>
+      <c r="G35" s="129"/>
+      <c r="H35" s="129"/>
+      <c r="I35" s="129"/>
+      <c r="J35" s="129"/>
+      <c r="K35" s="129"/>
+      <c r="L35" s="129"/>
+      <c r="M35" s="129"/>
+    </row>
+    <row r="36" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="123" t="s">
+        <v>440</v>
+      </c>
+      <c r="B36" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C36" s="54"/>
+      <c r="D36" s="129"/>
+      <c r="E36" s="129"/>
+      <c r="F36" s="129"/>
+      <c r="G36" s="129"/>
+      <c r="H36" s="129"/>
+      <c r="I36" s="129"/>
+      <c r="J36" s="129"/>
+      <c r="K36" s="129"/>
+      <c r="L36" s="129"/>
+      <c r="M36" s="129"/>
+    </row>
+    <row r="37" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="123" t="s">
+        <v>441</v>
+      </c>
+      <c r="B37" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C37" s="54"/>
+      <c r="D37" s="129"/>
+      <c r="E37" s="129"/>
+      <c r="F37" s="129"/>
+      <c r="G37" s="129"/>
+      <c r="H37" s="129"/>
+      <c r="I37" s="129"/>
+      <c r="J37" s="129"/>
+      <c r="K37" s="129"/>
+      <c r="L37" s="129"/>
+      <c r="M37" s="129"/>
+    </row>
+    <row r="38" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="123" t="s">
+        <v>442</v>
+      </c>
+      <c r="B38" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C38" s="54"/>
+      <c r="D38" s="129"/>
+      <c r="E38" s="129"/>
+      <c r="F38" s="129"/>
+      <c r="G38" s="129"/>
+      <c r="H38" s="129"/>
+      <c r="I38" s="129"/>
+      <c r="J38" s="129"/>
+      <c r="K38" s="129"/>
+      <c r="L38" s="129"/>
+      <c r="M38" s="129"/>
+    </row>
+    <row r="39" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="123" t="s">
+        <v>443</v>
+      </c>
+      <c r="B39" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C39" s="54"/>
+      <c r="D39" s="129"/>
+      <c r="E39" s="129"/>
+      <c r="F39" s="129"/>
+      <c r="G39" s="129"/>
+      <c r="H39" s="129"/>
+      <c r="I39" s="129"/>
+      <c r="J39" s="129"/>
+      <c r="K39" s="129"/>
+      <c r="L39" s="129"/>
+      <c r="M39" s="129"/>
+    </row>
+    <row r="40" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="123" t="s">
+        <v>444</v>
+      </c>
+      <c r="B40" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C40" s="54"/>
+      <c r="D40" s="129"/>
+      <c r="E40" s="129"/>
+      <c r="F40" s="129"/>
+      <c r="G40" s="129"/>
+      <c r="H40" s="129"/>
+      <c r="I40" s="129"/>
+      <c r="J40" s="129"/>
+      <c r="K40" s="129"/>
+      <c r="L40" s="129"/>
+      <c r="M40" s="129"/>
+    </row>
+    <row r="41" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="123" t="s">
+        <v>445</v>
+      </c>
+      <c r="B41" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C41" s="54"/>
+      <c r="D41" s="129"/>
+      <c r="E41" s="129"/>
+      <c r="F41" s="129"/>
+      <c r="G41" s="129"/>
+      <c r="H41" s="129"/>
+      <c r="I41" s="129"/>
+      <c r="J41" s="129"/>
+      <c r="K41" s="129"/>
+      <c r="L41" s="129"/>
+      <c r="M41" s="129"/>
+    </row>
+    <row r="42" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="123" t="s">
+        <v>446</v>
+      </c>
+      <c r="B42" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C42" s="54"/>
+      <c r="D42" s="129"/>
+      <c r="E42" s="129"/>
+      <c r="F42" s="129"/>
+      <c r="G42" s="129"/>
+      <c r="H42" s="129"/>
+      <c r="I42" s="129"/>
+      <c r="J42" s="129"/>
+      <c r="K42" s="129"/>
+      <c r="L42" s="129"/>
+      <c r="M42" s="129"/>
+    </row>
+    <row r="43" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="123" t="s">
+        <v>447</v>
+      </c>
+      <c r="B43" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C43" s="54"/>
+      <c r="D43" s="129"/>
+      <c r="E43" s="129"/>
+      <c r="F43" s="129"/>
+      <c r="G43" s="129"/>
+      <c r="H43" s="129"/>
+      <c r="I43" s="129"/>
+      <c r="J43" s="129"/>
+      <c r="K43" s="129"/>
+      <c r="L43" s="129"/>
+      <c r="M43" s="129"/>
+    </row>
+    <row r="44" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="123" t="s">
+        <v>448</v>
+      </c>
+      <c r="B44" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C44" s="54"/>
+      <c r="D44" s="129"/>
+      <c r="E44" s="129"/>
+      <c r="F44" s="129"/>
+      <c r="G44" s="129"/>
+      <c r="H44" s="129"/>
+      <c r="I44" s="129"/>
+      <c r="J44" s="129"/>
+      <c r="K44" s="129"/>
+      <c r="L44" s="129"/>
+      <c r="M44" s="129"/>
+    </row>
+    <row r="45" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="123" t="s">
+        <v>449</v>
+      </c>
+      <c r="B45" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C45" s="54"/>
+      <c r="D45" s="129"/>
+      <c r="E45" s="129"/>
+      <c r="F45" s="129"/>
+      <c r="G45" s="129"/>
+      <c r="H45" s="129"/>
+      <c r="I45" s="129"/>
+      <c r="J45" s="129"/>
+      <c r="K45" s="129"/>
+      <c r="L45" s="129"/>
+      <c r="M45" s="129"/>
+    </row>
+    <row r="46" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="123" t="s">
+        <v>450</v>
+      </c>
+      <c r="B46" s="130" t="s">
+        <v>385</v>
+      </c>
+      <c r="C46" s="54"/>
+      <c r="D46" s="129"/>
+      <c r="E46" s="129"/>
+      <c r="F46" s="129"/>
+      <c r="G46" s="129"/>
+      <c r="H46" s="129"/>
+      <c r="I46" s="129"/>
+      <c r="J46" s="129"/>
+      <c r="K46" s="129"/>
+      <c r="L46" s="129"/>
+      <c r="M46" s="129"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:J1"/>
   </mergeCells>
+  <phoneticPr fontId="13" type="noConversion"/>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="71" fitToHeight="0" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd"/>
@@ -5773,18 +6239,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="115" t="s">
         <v>330</v>
       </c>
-      <c r="B1" s="115"/>
-      <c r="C1" s="115"/>
-      <c r="D1" s="115"/>
-      <c r="E1" s="115"/>
-      <c r="F1" s="115"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
     </row>
     <row r="2" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="55" t="s">
@@ -5814,7 +6280,7 @@
       <c r="A3" s="16" t="s">
         <v>334</v>
       </c>
-      <c r="B3" s="63">
+      <c r="B3" s="62">
         <v>50</v>
       </c>
       <c r="C3" s="38">
@@ -5823,10 +6289,10 @@
       <c r="D3" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="63" t="s">
+      <c r="E3" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F3" s="63" t="s">
+      <c r="F3" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G3" s="4"/>
@@ -5838,7 +6304,7 @@
       <c r="A4" s="16" t="s">
         <v>335</v>
       </c>
-      <c r="B4" s="63">
+      <c r="B4" s="62">
         <v>55</v>
       </c>
       <c r="C4" s="38">
@@ -5847,10 +6313,10 @@
       <c r="D4" s="38" t="s">
         <v>302</v>
       </c>
-      <c r="E4" s="63" t="s">
+      <c r="E4" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F4" s="63" t="s">
+      <c r="F4" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G4" s="4"/>
@@ -5862,7 +6328,7 @@
       <c r="A5" s="16" t="s">
         <v>336</v>
       </c>
-      <c r="B5" s="63">
+      <c r="B5" s="62">
         <v>12</v>
       </c>
       <c r="C5" s="38">
@@ -5871,10 +6337,10 @@
       <c r="D5" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="63" t="s">
+      <c r="E5" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F5" s="63" t="s">
+      <c r="F5" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G5" s="4"/>
@@ -5886,7 +6352,7 @@
       <c r="A6" s="16" t="s">
         <v>337</v>
       </c>
-      <c r="B6" s="63">
+      <c r="B6" s="62">
         <v>43</v>
       </c>
       <c r="C6" s="38">
@@ -5895,10 +6361,10 @@
       <c r="D6" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="63" t="s">
+      <c r="E6" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F6" s="63" t="s">
+      <c r="F6" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G6" s="4"/>
@@ -5910,7 +6376,7 @@
       <c r="A7" s="16" t="s">
         <v>338</v>
       </c>
-      <c r="B7" s="63">
+      <c r="B7" s="62">
         <v>47</v>
       </c>
       <c r="C7" s="38">
@@ -5919,10 +6385,10 @@
       <c r="D7" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="63" t="s">
+      <c r="E7" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F7" s="63" t="s">
+      <c r="F7" s="62" t="s">
         <v>42</v>
       </c>
       <c r="G7" s="4"/>
@@ -5934,7 +6400,7 @@
       <c r="A8" s="16" t="s">
         <v>339</v>
       </c>
-      <c r="B8" s="63">
+      <c r="B8" s="62">
         <v>75</v>
       </c>
       <c r="C8" s="38">
@@ -5943,10 +6409,10 @@
       <c r="D8" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E8" s="63" t="s">
+      <c r="E8" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F8" s="63" t="s">
+      <c r="F8" s="62" t="s">
         <v>42</v>
       </c>
       <c r="G8" s="4"/>
@@ -5958,7 +6424,7 @@
       <c r="A9" s="16" t="s">
         <v>340</v>
       </c>
-      <c r="B9" s="63">
+      <c r="B9" s="62">
         <v>41</v>
       </c>
       <c r="C9" s="38">
@@ -5967,10 +6433,10 @@
       <c r="D9" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="63" t="s">
+      <c r="E9" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F9" s="63" t="s">
+      <c r="F9" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G9" s="4"/>
@@ -5982,7 +6448,7 @@
       <c r="A10" s="16" t="s">
         <v>341</v>
       </c>
-      <c r="B10" s="63">
+      <c r="B10" s="62">
         <v>15</v>
       </c>
       <c r="C10" s="38">
@@ -5991,10 +6457,10 @@
       <c r="D10" s="38" t="s">
         <v>302</v>
       </c>
-      <c r="E10" s="63" t="s">
+      <c r="E10" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F10" s="63" t="s">
+      <c r="F10" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G10" s="4"/>
@@ -6003,20 +6469,20 @@
       <c r="J10" s="4"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="66" t="s">
+      <c r="A11" s="65" t="s">
         <v>342</v>
       </c>
-      <c r="B11" s="67">
+      <c r="B11" s="66">
         <v>19</v>
       </c>
-      <c r="C11" s="68">
+      <c r="C11" s="67">
         <v>21</v>
       </c>
-      <c r="D11" s="68"/>
-      <c r="E11" s="67" t="s">
+      <c r="D11" s="67"/>
+      <c r="E11" s="66" t="s">
         <v>360</v>
       </c>
-      <c r="F11" s="67" t="s">
+      <c r="F11" s="66" t="s">
         <v>302</v>
       </c>
       <c r="G11" s="4"/>
@@ -6028,7 +6494,7 @@
       <c r="A12" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="B12" s="63">
+      <c r="B12" s="62">
         <v>24</v>
       </c>
       <c r="C12" s="38">
@@ -6037,10 +6503,10 @@
       <c r="D12" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="63" t="s">
+      <c r="E12" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F12" s="63" t="s">
+      <c r="F12" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G12" s="4"/>
@@ -6052,7 +6518,7 @@
       <c r="A13" s="16" t="s">
         <v>344</v>
       </c>
-      <c r="B13" s="63">
+      <c r="B13" s="62">
         <v>57</v>
       </c>
       <c r="C13" s="38">
@@ -6061,10 +6527,10 @@
       <c r="D13" s="38" t="s">
         <v>302</v>
       </c>
-      <c r="E13" s="63" t="s">
+      <c r="E13" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F13" s="63" t="s">
+      <c r="F13" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G13" s="4"/>
@@ -6076,19 +6542,19 @@
       <c r="A14" s="16" t="s">
         <v>345</v>
       </c>
-      <c r="B14" s="63">
+      <c r="B14" s="62">
         <v>37</v>
       </c>
-      <c r="C14" s="61">
+      <c r="C14" s="60">
         <v>56</v>
       </c>
       <c r="D14" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E14" s="63" t="s">
+      <c r="E14" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F14" s="63" t="s">
+      <c r="F14" s="62" t="s">
         <v>42</v>
       </c>
       <c r="G14" s="4"/>
@@ -6100,7 +6566,7 @@
       <c r="A15" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="B15" s="63">
+      <c r="B15" s="62">
         <v>53</v>
       </c>
       <c r="C15" s="38">
@@ -6109,10 +6575,10 @@
       <c r="D15" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="63" t="s">
+      <c r="E15" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F15" s="63" t="s">
+      <c r="F15" s="62" t="s">
         <v>42</v>
       </c>
       <c r="G15" s="4"/>
@@ -6124,7 +6590,7 @@
       <c r="A16" s="16" t="s">
         <v>347</v>
       </c>
-      <c r="B16" s="63">
+      <c r="B16" s="62">
         <v>60</v>
       </c>
       <c r="C16" s="38">
@@ -6133,10 +6599,10 @@
       <c r="D16" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E16" s="63" t="s">
+      <c r="E16" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F16" s="63" t="s">
+      <c r="F16" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G16" s="4"/>
@@ -6148,7 +6614,7 @@
       <c r="A17" s="16" t="s">
         <v>348</v>
       </c>
-      <c r="B17" s="63">
+      <c r="B17" s="62">
         <v>45</v>
       </c>
       <c r="C17" s="38">
@@ -6157,10 +6623,10 @@
       <c r="D17" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="63" t="s">
+      <c r="E17" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F17" s="63" t="s">
+      <c r="F17" s="62" t="s">
         <v>42</v>
       </c>
       <c r="G17" s="4"/>
@@ -6169,22 +6635,22 @@
       <c r="J17" s="4"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="96" t="s">
+      <c r="A18" s="95" t="s">
         <v>349</v>
       </c>
-      <c r="B18" s="97">
+      <c r="B18" s="96">
         <v>16</v>
       </c>
-      <c r="C18" s="98">
+      <c r="C18" s="97">
         <v>17</v>
       </c>
-      <c r="D18" s="98" t="s">
+      <c r="D18" s="97" t="s">
         <v>42</v>
       </c>
-      <c r="E18" s="97" t="s">
+      <c r="E18" s="96" t="s">
         <v>360</v>
       </c>
-      <c r="F18" s="97" t="s">
+      <c r="F18" s="96" t="s">
         <v>302</v>
       </c>
       <c r="G18" s="4"/>
@@ -6196,7 +6662,7 @@
       <c r="A19" s="16" t="s">
         <v>350</v>
       </c>
-      <c r="B19" s="63" t="s">
+      <c r="B19" s="62" t="s">
         <v>361</v>
       </c>
       <c r="C19" s="38" t="s">
@@ -6205,10 +6671,10 @@
       <c r="D19" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="63" t="s">
+      <c r="E19" s="62" t="s">
         <v>363</v>
       </c>
-      <c r="F19" s="63" t="s">
+      <c r="F19" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G19" s="4"/>
@@ -6220,19 +6686,19 @@
       <c r="A20" s="16" t="s">
         <v>351</v>
       </c>
-      <c r="B20" s="63">
+      <c r="B20" s="62">
         <v>18</v>
       </c>
-      <c r="C20" s="61">
+      <c r="C20" s="60">
         <v>40</v>
       </c>
       <c r="D20" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="63" t="s">
+      <c r="E20" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F20" s="63" t="s">
+      <c r="F20" s="62" t="s">
         <v>42</v>
       </c>
       <c r="G20" s="4"/>
@@ -6244,7 +6710,7 @@
       <c r="A21" s="16" t="s">
         <v>352</v>
       </c>
-      <c r="B21" s="63">
+      <c r="B21" s="62">
         <v>34</v>
       </c>
       <c r="C21" s="38">
@@ -6253,10 +6719,10 @@
       <c r="D21" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E21" s="63" t="s">
+      <c r="E21" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F21" s="63" t="s">
+      <c r="F21" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G21" s="4"/>
@@ -6265,22 +6731,22 @@
       <c r="J21" s="4"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" s="95" t="s">
+      <c r="A22" s="94" t="s">
         <v>353</v>
       </c>
-      <c r="B22" s="63">
+      <c r="B22" s="62">
         <v>83</v>
       </c>
-      <c r="C22" s="61">
+      <c r="C22" s="60">
         <v>84</v>
       </c>
       <c r="D22" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E22" s="63" t="s">
+      <c r="E22" s="62" t="s">
         <v>360</v>
       </c>
-      <c r="F22" s="63" t="s">
+      <c r="F22" s="62" t="s">
         <v>302</v>
       </c>
       <c r="G22" s="4"/>
@@ -6289,22 +6755,22 @@
       <c r="J22" s="4"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" s="88" t="s">
+      <c r="A23" s="87" t="s">
         <v>354</v>
       </c>
-      <c r="B23" s="89" t="s">
+      <c r="B23" s="88" t="s">
         <v>375</v>
       </c>
-      <c r="C23" s="90" t="s">
+      <c r="C23" s="89" t="s">
         <v>376</v>
       </c>
-      <c r="D23" s="91" t="s">
+      <c r="D23" s="90" t="s">
         <v>42</v>
       </c>
-      <c r="E23" s="89" t="s">
+      <c r="E23" s="88" t="s">
         <v>363</v>
       </c>
-      <c r="F23" s="89" t="s">
+      <c r="F23" s="88" t="s">
         <v>302</v>
       </c>
       <c r="G23" s="4"/>
@@ -6313,22 +6779,22 @@
       <c r="J23" s="4"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="88" t="s">
+      <c r="A24" s="87" t="s">
         <v>355</v>
       </c>
-      <c r="B24" s="89" t="s">
+      <c r="B24" s="88" t="s">
         <v>377</v>
       </c>
-      <c r="C24" s="90" t="s">
+      <c r="C24" s="89" t="s">
         <v>378</v>
       </c>
-      <c r="D24" s="91" t="s">
+      <c r="D24" s="90" t="s">
         <v>42</v>
       </c>
-      <c r="E24" s="89" t="s">
+      <c r="E24" s="88" t="s">
         <v>363</v>
       </c>
-      <c r="F24" s="89" t="s">
+      <c r="F24" s="88" t="s">
         <v>302</v>
       </c>
       <c r="G24" s="4"/>
@@ -6337,22 +6803,22 @@
       <c r="J24" s="4"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="88" t="s">
+      <c r="A25" s="87" t="s">
         <v>356</v>
       </c>
-      <c r="B25" s="89" t="s">
+      <c r="B25" s="88" t="s">
         <v>383</v>
       </c>
-      <c r="C25" s="90" t="s">
+      <c r="C25" s="89" t="s">
         <v>384</v>
       </c>
-      <c r="D25" s="91" t="s">
+      <c r="D25" s="90" t="s">
         <v>42</v>
       </c>
-      <c r="E25" s="89" t="s">
+      <c r="E25" s="88" t="s">
         <v>363</v>
       </c>
-      <c r="F25" s="89" t="s">
+      <c r="F25" s="88" t="s">
         <v>302</v>
       </c>
       <c r="G25" s="4"/>
@@ -6361,47 +6827,47 @@
       <c r="J25" s="4"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="88" t="s">
+      <c r="A26" s="87" t="s">
         <v>357</v>
       </c>
-      <c r="B26" s="89">
+      <c r="B26" s="88">
         <v>30</v>
       </c>
-      <c r="C26" s="90">
+      <c r="C26" s="89">
         <v>68</v>
       </c>
-      <c r="D26" s="91" t="s">
+      <c r="D26" s="90" t="s">
         <v>42</v>
       </c>
-      <c r="E26" s="89" t="s">
+      <c r="E26" s="88" t="s">
         <v>360</v>
       </c>
-      <c r="F26" s="89" t="s">
+      <c r="F26" s="88" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="88" t="s">
+      <c r="A27" s="87" t="s">
         <v>358</v>
       </c>
-      <c r="B27" s="89">
+      <c r="B27" s="88">
         <v>3</v>
       </c>
-      <c r="C27" s="90">
+      <c r="C27" s="89">
         <v>2</v>
       </c>
-      <c r="D27" s="91" t="s">
+      <c r="D27" s="90" t="s">
         <v>42</v>
       </c>
-      <c r="E27" s="89" t="s">
+      <c r="E27" s="88" t="s">
         <v>360</v>
       </c>
-      <c r="F27" s="89" t="s">
+      <c r="F27" s="88" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="122" t="s">
+      <c r="A29" s="104" t="s">
         <v>425</v>
       </c>
       <c r="B29" s="33" t="s">
@@ -6410,7 +6876,7 @@
       <c r="C29" s="33" t="s">
         <v>429</v>
       </c>
-      <c r="E29" s="123" t="s">
+      <c r="E29" s="105" t="s">
         <v>431</v>
       </c>
       <c r="G29" s="33" t="s">
@@ -6418,7 +6884,7 @@
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" s="122" t="s">
+      <c r="A30" s="104" t="s">
         <v>426</v>
       </c>
       <c r="B30" s="33" t="s">
@@ -6427,7 +6893,7 @@
       <c r="C30" s="33" t="s">
         <v>428</v>
       </c>
-      <c r="E30" s="123" t="s">
+      <c r="E30" s="105" t="s">
         <v>431</v>
       </c>
       <c r="G30" s="33" t="s">
@@ -6455,20 +6921,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="117" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="116" t="s">
+      <c r="B1" s="118"/>
+      <c r="C1" s="117" t="s">
         <v>251</v>
       </c>
-      <c r="D1" s="118"/>
-      <c r="E1" s="118"/>
-      <c r="F1" s="118"/>
-      <c r="G1" s="118"/>
-      <c r="H1" s="118"/>
-      <c r="I1" s="118"/>
-      <c r="J1" s="117"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="118"/>
     </row>
     <row r="2" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="37" t="s">
@@ -6654,7 +7120,7 @@
       <c r="A11" s="26" t="s">
         <v>243</v>
       </c>
-      <c r="B11" s="60" t="s">
+      <c r="B11" s="59" t="s">
         <v>413</v>
       </c>
       <c r="C11" s="32" t="s">
@@ -6770,7 +7236,7 @@
       <c r="A17" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="B17" s="60" t="s">
+      <c r="B17" s="59" t="s">
         <v>315</v>
       </c>
       <c r="C17" s="34" t="s">
@@ -6790,7 +7256,7 @@
       <c r="A18" s="29" t="s">
         <v>132</v>
       </c>
-      <c r="B18" s="60" t="s">
+      <c r="B18" s="59" t="s">
         <v>237</v>
       </c>
       <c r="C18" s="34" t="s">
@@ -6810,7 +7276,7 @@
       <c r="A19" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="B19" s="60" t="s">
+      <c r="B19" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C19" s="34" t="s">
@@ -6830,7 +7296,7 @@
       <c r="A20" s="28" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="94" t="s">
+      <c r="B20" s="93" t="s">
         <v>235</v>
       </c>
       <c r="C20" s="36" t="s">
@@ -6968,7 +7434,7 @@
       <c r="A28" s="28" t="s">
         <v>407</v>
       </c>
-      <c r="B28" s="93" t="s">
+      <c r="B28" s="92" t="s">
         <v>126</v>
       </c>
       <c r="C28" s="36" t="s">
@@ -7026,30 +7492,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="120" t="s">
         <v>297</v>
       </c>
-      <c r="B1" s="120"/>
-      <c r="C1" s="120"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="109" t="s">
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="110" t="s">
         <v>397</v>
       </c>
-      <c r="F1" s="109"/>
-      <c r="G1" s="109"/>
-      <c r="H1" s="121" t="s">
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="122" t="s">
         <v>410</v>
       </c>
-      <c r="I1" s="121"/>
+      <c r="I1" s="122"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="83" t="s">
+      <c r="A2" s="82" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="83" t="s">
+      <c r="B2" s="82" t="s">
         <v>299</v>
       </c>
-      <c r="C2" s="83" t="s">
+      <c r="C2" s="82" t="s">
         <v>298</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -7069,14 +7535,14 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="85" t="str">
+      <c r="A3" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1h79fqthLoRJDjhC2klnjbkG8MB2JL2Hy","1A")</f>
         <v>1A</v>
       </c>
       <c r="B3" s="52" t="s">
         <v>300</v>
       </c>
-      <c r="C3" s="84" t="s">
+      <c r="C3" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D3" s="54" t="s">
@@ -7085,25 +7551,25 @@
       <c r="E3" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="74" t="s">
+      <c r="F3" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="73" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="85" t="str">
+      <c r="A4" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1OPl2VmHH1ZeMZjQWNCCkQkA6bOfyIeqj","1B")</f>
         <v>1B</v>
       </c>
       <c r="B4" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C4" s="84" t="s">
+      <c r="C4" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D4" s="54" t="s">
@@ -7112,23 +7578,23 @@
       <c r="E4" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H4" s="74" t="s">
+      <c r="F4" s="72"/>
+      <c r="G4" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="86" t="str">
+      <c r="A5" s="85" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1_67Lwh4ATjaUkKTpdhqNA2vhhSxMhfoh","1C")</f>
         <v>1C</v>
       </c>
       <c r="B5" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C5" s="84" t="s">
+      <c r="C5" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D5" s="54" t="s">
@@ -7140,22 +7606,22 @@
       <c r="F5" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" s="74" t="s">
+      <c r="G5" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="86" t="str">
+      <c r="A6" s="85" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1RDZathABUe1AxNllos18oBRUGkUw-BAb","1D")</f>
         <v>1D</v>
       </c>
       <c r="B6" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C6" s="84" t="s">
+      <c r="C6" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D6" s="54" t="s">
@@ -7164,23 +7630,23 @@
       <c r="E6" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="73"/>
-      <c r="G6" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6" s="74" t="s">
+      <c r="F6" s="72"/>
+      <c r="G6" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="86" t="str">
+      <c r="A7" s="85" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1B7jEgQfvgjZIKbfW8eR9qm2PDLYRcFFX","1E")</f>
         <v>1E</v>
       </c>
       <c r="B7" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C7" s="84" t="s">
+      <c r="C7" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D7" s="54" t="s">
@@ -7192,22 +7658,22 @@
       <c r="F7" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H7" s="74" t="s">
+      <c r="G7" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="86" t="str">
+      <c r="A8" s="85" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1y8psJsldf8GOPKXdI3_7jAN-0VefmuVb","1F")</f>
         <v>1F</v>
       </c>
       <c r="B8" s="52" t="s">
         <v>300</v>
       </c>
-      <c r="C8" s="84" t="s">
+      <c r="C8" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D8" s="54" t="s">
@@ -7216,25 +7682,25 @@
       <c r="E8" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H8" s="74" t="s">
+      <c r="F8" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="73" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="85" t="str">
+      <c r="A9" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1Ak0bagtonjeBe0T45ml7mh9V5vKH_FoI","1G")</f>
         <v>1G</v>
       </c>
       <c r="B9" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C9" s="84" t="s">
+      <c r="C9" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D9" s="54" t="s">
@@ -7246,22 +7712,22 @@
       <c r="F9" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H9" s="74" t="s">
+      <c r="G9" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="85" t="str">
+      <c r="A10" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=15tp_vGgbK5-4zzthz0W8wuq2zgKokja6","1H")</f>
         <v>1H</v>
       </c>
       <c r="B10" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C10" s="84" t="s">
+      <c r="C10" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D10" s="54" t="s">
@@ -7270,25 +7736,25 @@
       <c r="E10" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H10" s="74" t="s">
+      <c r="F10" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="85" t="str">
+      <c r="A11" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1EMft8Du0dvrSSlstsShqV16Nnrlb4EO_","1J")</f>
         <v>1J</v>
       </c>
       <c r="B11" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C11" s="84" t="s">
+      <c r="C11" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D11" s="54" t="s">
@@ -7298,22 +7764,22 @@
         <v>25</v>
       </c>
       <c r="F11" s="54"/>
-      <c r="G11" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H11" s="74" t="s">
+      <c r="G11" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="85" t="str">
+      <c r="A12" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1B-AwkTkUdHQS0dThuP6mM5L_0XIFZ2QS","1K")</f>
         <v>1K</v>
       </c>
       <c r="B12" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C12" s="84" t="s">
+      <c r="C12" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D12" s="54" t="s">
@@ -7322,25 +7788,25 @@
       <c r="E12" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G12" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H12" s="74" t="s">
+      <c r="F12" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="85" t="str">
+      <c r="A13" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1XILFfrJerwAeHeN4xKdQH-99VN9y0QS7","2A")</f>
         <v>2A</v>
       </c>
       <c r="B13" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C13" s="84" t="s">
+      <c r="C13" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D13" s="54" t="s">
@@ -7349,25 +7815,25 @@
       <c r="E13" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G13" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H13" s="74" t="s">
+      <c r="F13" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="85" t="str">
+      <c r="A14" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1i7lErxBcw13LxRubiAB_0upxTGrTLBvi","2B")</f>
         <v>2B</v>
       </c>
       <c r="B14" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C14" s="84" t="s">
+      <c r="C14" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D14" s="54" t="s">
@@ -7376,25 +7842,25 @@
       <c r="E14" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F14" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G14" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H14" s="74" t="s">
+      <c r="F14" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H14" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="85" t="str">
+      <c r="A15" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1HmSkhlRiy_w_xIcPrlD-Gu21Q1sHCajk","2C")</f>
         <v>2C</v>
       </c>
       <c r="B15" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C15" s="84" t="s">
+      <c r="C15" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D15" s="54" t="s">
@@ -7403,25 +7869,25 @@
       <c r="E15" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F15" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H15" s="74" t="s">
+      <c r="F15" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="85" t="str">
+      <c r="A16" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1ih9AM9nSu6WpURV8EnXu6Q1HkOh5dSXM","2D")</f>
         <v>2D</v>
       </c>
       <c r="B16" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C16" s="84" t="s">
+      <c r="C16" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D16" s="54" t="s">
@@ -7430,23 +7896,23 @@
       <c r="E16" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F16" s="73"/>
-      <c r="G16" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H16" s="74" t="s">
+      <c r="F16" s="72"/>
+      <c r="G16" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H16" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="85" t="str">
+      <c r="A17" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1ilbwUzFLn2Zr9CQ_v673T9KjSALf_GzB","2E")</f>
         <v>2E</v>
       </c>
       <c r="B17" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C17" s="84" t="s">
+      <c r="C17" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D17" s="54" t="s">
@@ -7455,25 +7921,25 @@
       <c r="E17" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F17" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G17" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H17" s="74" t="s">
+      <c r="F17" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G17" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="85" t="str">
+      <c r="A18" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1H2B7fJmOymk8ZeyITqVgqJIR9EbewGjs","2F")</f>
         <v>2F</v>
       </c>
       <c r="B18" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C18" s="84" t="s">
+      <c r="C18" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D18" s="54" t="s">
@@ -7482,23 +7948,23 @@
       <c r="E18" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F18" s="73"/>
-      <c r="G18" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H18" s="74" t="s">
+      <c r="F18" s="72"/>
+      <c r="G18" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H18" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="85" t="str">
+      <c r="A19" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1GXDi1coA9HtIo5F2GTLcPhpAh_IiHrmJ","2G")</f>
         <v>2G</v>
       </c>
       <c r="B19" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C19" s="84" t="s">
+      <c r="C19" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D19" s="54" t="s">
@@ -7508,22 +7974,22 @@
         <v>25</v>
       </c>
       <c r="F19" s="54"/>
-      <c r="G19" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H19" s="74" t="s">
+      <c r="G19" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H19" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="85" t="str">
+      <c r="A20" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=18itspidwzvb4KFHkqj1122TxuhHxILwX","2H")</f>
         <v>2H</v>
       </c>
       <c r="B20" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C20" s="84" t="s">
+      <c r="C20" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D20" s="54" t="s">
@@ -7532,25 +7998,25 @@
       <c r="E20" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G20" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H20" s="74" t="s">
+      <c r="F20" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G20" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H20" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="85" t="str">
+      <c r="A21" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=12YgGEJrua5a-agu15lV4vezflw1cOjQ4","2J")</f>
         <v>2J</v>
       </c>
       <c r="B21" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C21" s="84" t="s">
+      <c r="C21" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D21" s="54" t="s">
@@ -7559,25 +8025,25 @@
       <c r="E21" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F21" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G21" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H21" s="74" t="s">
+      <c r="F21" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G21" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H21" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="85" t="str">
+      <c r="A22" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1mdMrKj4CCNPy7BlChSDOU2hQAJONhZzU","2K")</f>
         <v>2K</v>
       </c>
       <c r="B22" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C22" s="84" t="s">
+      <c r="C22" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D22" s="54" t="s">
@@ -7586,25 +8052,25 @@
       <c r="E22" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F22" s="74" t="s">
-        <v>25</v>
-      </c>
-      <c r="G22" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H22" s="74" t="s">
+      <c r="F22" s="73" t="s">
+        <v>25</v>
+      </c>
+      <c r="G22" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H22" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="85" t="str">
+      <c r="A23" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=14mzIl-szkFL_WWXlsFZ9T_x3Mt5RAOn0","2L")</f>
         <v>2L</v>
       </c>
       <c r="B23" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C23" s="84" t="s">
+      <c r="C23" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D23" s="54" t="s">
@@ -7613,25 +8079,25 @@
       <c r="E23" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G23" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H23" s="74" t="s">
+      <c r="F23" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G23" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H23" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="85" t="str">
+      <c r="A24" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1-X_VRvOqUUm_bcQ792NJw8TTxR5Kl3lr","2M")</f>
         <v>2M</v>
       </c>
       <c r="B24" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C24" s="84" t="s">
+      <c r="C24" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D24" s="54" t="s">
@@ -7643,22 +8109,22 @@
       <c r="F24" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="G24" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H24" s="74" t="s">
+      <c r="G24" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H24" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="85" t="str">
+      <c r="A25" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1ofYuI7zJYOx0Em5kOgymDe9L2TWaIZ-_","3C")</f>
         <v>3C</v>
       </c>
       <c r="B25" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C25" s="84" t="s">
+      <c r="C25" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D25" s="54" t="s">
@@ -7667,25 +8133,25 @@
       <c r="E25" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F25" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G25" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H25" s="74" t="s">
+      <c r="F25" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G25" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H25" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="85" t="str">
+      <c r="A26" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1X9eTLHcdh-lSX2OXG4OLDNwPRG5eoz9l","3D")</f>
         <v>3D</v>
       </c>
       <c r="B26" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C26" s="84" t="s">
+      <c r="C26" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D26" s="54" t="s">
@@ -7697,22 +8163,22 @@
       <c r="F26" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="G26" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H26" s="74" t="s">
+      <c r="G26" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H26" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="85" t="str">
+      <c r="A27" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1m_ACLfEw9sFFcCd16wQnkI9wa3WI7gK9","3E")</f>
         <v>3E</v>
       </c>
       <c r="B27" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C27" s="84" t="s">
+      <c r="C27" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D27" s="54" t="s">
@@ -7721,78 +8187,78 @@
       <c r="E27" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F27" s="73"/>
-      <c r="G27" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H27" s="74" t="s">
+      <c r="F27" s="72"/>
+      <c r="G27" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H27" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" s="85" t="str">
+      <c r="A28" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1CIBdXiHhWBrM6LwlY-yGooPill1DRTQ7","3F")</f>
         <v>3F</v>
       </c>
-      <c r="B28" s="92" t="s">
+      <c r="B28" s="91" t="s">
         <v>42</v>
       </c>
-      <c r="C28" s="84" t="s">
+      <c r="C28" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D28" s="54"/>
       <c r="E28" s="54"/>
       <c r="F28" s="54"/>
-      <c r="G28" s="73"/>
-      <c r="H28" s="73"/>
+      <c r="G28" s="72"/>
+      <c r="H28" s="72"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="85" t="str">
+      <c r="A29" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1c2xmouFbs4cNAvpeHuAdgNreh8kFEC2V","3G")</f>
         <v>3G</v>
       </c>
-      <c r="B29" s="92" t="s">
+      <c r="B29" s="91" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="84" t="s">
+      <c r="C29" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D29" s="54"/>
       <c r="E29" s="54"/>
       <c r="F29" s="54"/>
-      <c r="G29" s="73"/>
-      <c r="H29" s="74" t="s">
+      <c r="G29" s="72"/>
+      <c r="H29" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="85" t="str">
+      <c r="A30" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1t7wkFvS4sGjdMU60zYacdFSrl4pYayl_","3H")</f>
         <v>3H</v>
       </c>
-      <c r="B30" s="92" t="s">
+      <c r="B30" s="91" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="84" t="s">
+      <c r="C30" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D30" s="54"/>
       <c r="E30" s="54"/>
       <c r="F30" s="54"/>
-      <c r="G30" s="73"/>
-      <c r="H30" s="74" t="s">
+      <c r="G30" s="72"/>
+      <c r="H30" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" s="85" t="str">
+      <c r="A31" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1N0-R1KTkpoZjXWmN7r0U_myR9XBY5SDj","3J")</f>
         <v>3J</v>
       </c>
       <c r="B31" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C31" s="84" t="s">
+      <c r="C31" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D31" s="54" t="s">
@@ -7801,23 +8267,23 @@
       <c r="E31" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F31" s="73"/>
-      <c r="G31" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H31" s="74" t="s">
+      <c r="F31" s="72"/>
+      <c r="G31" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H31" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="85" t="str">
+      <c r="A32" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=13pmWKIsTMFsSuBTJ-HZb5DVIowIXTS_s","3L")</f>
         <v>3L</v>
       </c>
       <c r="B32" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C32" s="84" t="s">
+      <c r="C32" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D32" s="54" t="s">
@@ -7826,25 +8292,25 @@
       <c r="E32" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F32" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G32" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H32" s="74" t="s">
+      <c r="F32" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G32" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H32" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="85" t="str">
+      <c r="A33" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=16nGNQgv2r19h9agxYjXmQ8rC4v330dYf","4E")</f>
         <v>4E</v>
       </c>
       <c r="B33" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C33" s="84" t="s">
+      <c r="C33" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D33" s="54" t="s">
@@ -7856,22 +8322,22 @@
       <c r="F33" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="G33" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H33" s="74" t="s">
+      <c r="G33" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H33" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="85" t="str">
+      <c r="A34" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1bmJc7h6PrfobWHjtATEPhVDZqxi3ORaa","4F")</f>
         <v>4F</v>
       </c>
       <c r="B34" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C34" s="84" t="s">
+      <c r="C34" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D34" s="54" t="s">
@@ -7881,22 +8347,22 @@
         <v>25</v>
       </c>
       <c r="F34" s="54"/>
-      <c r="G34" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H34" s="74" t="s">
+      <c r="G34" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H34" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="85" t="str">
+      <c r="A35" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1nHAP6VZOPX4PWClDeQpEHh4MuzIQchEa","4G")</f>
         <v>4G</v>
       </c>
       <c r="B35" s="52" t="s">
         <v>300</v>
       </c>
-      <c r="C35" s="84" t="s">
+      <c r="C35" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D35" s="54" t="s">
@@ -7905,25 +8371,25 @@
       <c r="E35" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F35" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G35" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H35" s="74" t="s">
+      <c r="F35" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G35" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H35" s="73" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="85" t="str">
+      <c r="A36" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1a78u8iOyRFbuJtQlj9X51FknS9EfCDih","4H")</f>
         <v>4H</v>
       </c>
       <c r="B36" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C36" s="84" t="s">
+      <c r="C36" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D36" s="54" t="s">
@@ -7933,22 +8399,22 @@
         <v>25</v>
       </c>
       <c r="F36" s="54"/>
-      <c r="G36" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H36" s="74" t="s">
+      <c r="G36" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H36" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="85" t="str">
+      <c r="A37" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1zZjefBVzFC9BP-YmMKfQZMWa1XGkqomj","4J")</f>
         <v>4J</v>
       </c>
       <c r="B37" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C37" s="84" t="s">
+      <c r="C37" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D37" s="54" t="s">
@@ -7957,25 +8423,25 @@
       <c r="E37" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F37" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G37" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H37" s="74" t="s">
+      <c r="F37" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G37" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H37" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38" s="85" t="str">
+      <c r="A38" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1qWFlabv0TeVOBvOIJQuvHlR1H3AMOPvN","4K")</f>
         <v>4K</v>
       </c>
       <c r="B38" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C38" s="84" t="s">
+      <c r="C38" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D38" s="54" t="s">
@@ -7984,23 +8450,23 @@
       <c r="E38" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F38" s="73"/>
-      <c r="G38" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H38" s="74" t="s">
+      <c r="F38" s="72"/>
+      <c r="G38" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H38" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39" s="85" t="str">
+      <c r="A39" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=176NV2NM9yvfuW1EMU3iBS768FxgmXjUS","4L")</f>
         <v>4L</v>
       </c>
       <c r="B39" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C39" s="84" t="s">
+      <c r="C39" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D39" s="54" t="s">
@@ -8009,23 +8475,23 @@
       <c r="E39" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F39" s="73"/>
-      <c r="G39" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H39" s="74" t="s">
+      <c r="F39" s="72"/>
+      <c r="G39" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H39" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="85" t="str">
+      <c r="A40" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1cC0P-G66cPSNnf6v6z8opZCNyporo74Y","5B")</f>
         <v>5B</v>
       </c>
       <c r="B40" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C40" s="84" t="s">
+      <c r="C40" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D40" s="54" t="s">
@@ -8034,25 +8500,25 @@
       <c r="E40" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F40" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G40" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H40" s="74" t="s">
+      <c r="F40" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G40" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H40" s="73" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" s="85" t="str">
+      <c r="A41" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1q_N74b1OZrCze7zuXy5fm0ASU07tWzh3","5C")</f>
         <v>5C</v>
       </c>
       <c r="B41" s="52" t="s">
         <v>300</v>
       </c>
-      <c r="C41" s="84" t="s">
+      <c r="C41" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D41" s="54" t="s">
@@ -8061,25 +8527,25 @@
       <c r="E41" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F41" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="G41" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H41" s="74" t="s">
+      <c r="F41" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="G41" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H41" s="73" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="85" t="str">
+      <c r="A42" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1aKSCelAY002Ihje9mdJi7jFh0OB4j8XZ","5E")</f>
         <v>5E</v>
       </c>
       <c r="B42" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C42" s="84" t="s">
+      <c r="C42" s="83" t="s">
         <v>302</v>
       </c>
       <c r="D42" s="54" t="s">
@@ -8088,23 +8554,23 @@
       <c r="E42" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F42" s="73"/>
-      <c r="G42" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H42" s="74" t="s">
+      <c r="F42" s="72"/>
+      <c r="G42" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H42" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="85" t="str">
+      <c r="A43" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1ghdX_COwJq4oYlhj-qYPypK_2GlrWyQZ","5G")</f>
         <v>5G</v>
       </c>
       <c r="B43" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C43" s="84" t="s">
+      <c r="C43" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D43" s="54" t="s">
@@ -8113,23 +8579,23 @@
       <c r="E43" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F43" s="73"/>
-      <c r="G43" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H43" s="74" t="s">
+      <c r="F43" s="72"/>
+      <c r="G43" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H43" s="73" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44" s="85" t="str">
+      <c r="A44" s="84" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1MR24L4GDI5x861k8SMrgm71xRfm55Hiv","5H")</f>
         <v>5H</v>
       </c>
       <c r="B44" s="53" t="s">
         <v>301</v>
       </c>
-      <c r="C44" s="84" t="s">
+      <c r="C44" s="83" t="s">
         <v>42</v>
       </c>
       <c r="D44" s="54" t="s">
@@ -8138,11 +8604,11 @@
       <c r="E44" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="F44" s="73"/>
-      <c r="G44" s="73" t="s">
-        <v>25</v>
-      </c>
-      <c r="H44" s="74" t="s">
+      <c r="F44" s="72"/>
+      <c r="G44" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="H44" s="73" t="s">
         <v>25</v>
       </c>
     </row>
@@ -8176,30 +8642,30 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="68" t="s">
         <v>126</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="68" t="s">
         <v>379</v>
       </c>
-      <c r="C3" s="69" t="s">
+      <c r="C3" s="68" t="s">
         <v>380</v>
       </c>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
     </row>
     <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="69" t="s">
+      <c r="A4" s="68" t="s">
         <v>126</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="68" t="s">
         <v>149</v>
       </c>
-      <c r="C4" s="69" t="s">
+      <c r="C4" s="68" t="s">
         <v>150</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
       <c r="G4" t="s">
         <v>409</v>
       </c>
@@ -8210,73 +8676,73 @@
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="64" t="s">
+      <c r="A6" s="63" t="s">
         <v>357</v>
       </c>
-      <c r="B6" s="64" t="s">
+      <c r="B6" s="63" t="s">
         <v>143</v>
       </c>
-      <c r="C6" s="65"/>
-      <c r="D6" s="65"/>
-      <c r="E6" s="65" t="s">
+      <c r="C6" s="64"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="64" t="s">
+      <c r="A7" s="63" t="s">
         <v>357</v>
       </c>
-      <c r="B7" s="64" t="s">
+      <c r="B7" s="63" t="s">
         <v>144</v>
       </c>
-      <c r="C7" s="65"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="65" t="s">
+      <c r="C7" s="64"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="64" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="64" t="s">
+      <c r="A8" s="63" t="s">
         <v>342</v>
       </c>
-      <c r="B8" s="64" t="s">
+      <c r="B8" s="63" t="s">
         <v>145</v>
       </c>
-      <c r="C8" s="64" t="s">
+      <c r="C8" s="63" t="s">
         <v>146</v>
       </c>
-      <c r="D8" s="65"/>
-      <c r="E8" s="65" t="s">
+      <c r="D8" s="64"/>
+      <c r="E8" s="64" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="64" t="s">
+      <c r="A9" s="63" t="s">
         <v>342</v>
       </c>
-      <c r="B9" s="64" t="s">
+      <c r="B9" s="63" t="s">
         <v>147</v>
       </c>
-      <c r="C9" s="64" t="s">
+      <c r="C9" s="63" t="s">
         <v>146</v>
       </c>
-      <c r="D9" s="65"/>
-      <c r="E9" s="65" t="s">
+      <c r="D9" s="64"/>
+      <c r="E9" s="64" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="64" t="s">
+      <c r="A11" s="63" t="s">
         <v>126</v>
       </c>
-      <c r="B11" s="64" t="s">
+      <c r="B11" s="63" t="s">
         <v>148</v>
       </c>
-      <c r="C11" s="64" t="s">
+      <c r="C11" s="63" t="s">
         <v>386</v>
       </c>
-      <c r="D11" s="65"/>
-      <c r="E11" s="64" t="s">
+      <c r="D11" s="64"/>
+      <c r="E11" s="63" t="s">
         <v>142</v>
       </c>
     </row>
@@ -8287,17 +8753,17 @@
       <c r="C13" s="3"/>
     </row>
     <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="71" t="s">
+      <c r="A14" s="70" t="s">
         <v>126</v>
       </c>
-      <c r="B14" s="71" t="s">
+      <c r="B14" s="70" t="s">
         <v>291</v>
       </c>
-      <c r="C14" s="71" t="s">
+      <c r="C14" s="70" t="s">
         <v>293</v>
       </c>
-      <c r="D14" s="72"/>
-      <c r="E14" s="72"/>
+      <c r="D14" s="71"/>
+      <c r="E14" s="71"/>
     </row>
     <row r="15" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
@@ -8317,32 +8783,32 @@
       <c r="C16" s="3"/>
     </row>
     <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="64" t="s">
+      <c r="A17" s="63" t="s">
         <v>356</v>
       </c>
-      <c r="B17" s="64" t="s">
+      <c r="B17" s="63" t="s">
         <v>305</v>
       </c>
-      <c r="C17" s="64" t="s">
+      <c r="C17" s="63" t="s">
         <v>382</v>
       </c>
-      <c r="D17" s="65"/>
-      <c r="E17" s="64" t="s">
+      <c r="D17" s="64"/>
+      <c r="E17" s="63" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="64" t="s">
+      <c r="A18" s="63" t="s">
         <v>356</v>
       </c>
-      <c r="B18" s="64" t="s">
+      <c r="B18" s="63" t="s">
         <v>295</v>
       </c>
-      <c r="C18" s="64" t="s">
+      <c r="C18" s="63" t="s">
         <v>382</v>
       </c>
-      <c r="D18" s="65"/>
-      <c r="E18" s="64" t="s">
+      <c r="D18" s="64"/>
+      <c r="E18" s="63" t="s">
         <v>142</v>
       </c>
     </row>
@@ -8352,32 +8818,32 @@
       <c r="C19" s="3"/>
     </row>
     <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="64" t="s">
+      <c r="A20" s="63" t="s">
         <v>358</v>
       </c>
-      <c r="B20" s="64" t="s">
+      <c r="B20" s="63" t="s">
         <v>294</v>
       </c>
-      <c r="C20" s="64" t="s">
+      <c r="C20" s="63" t="s">
         <v>381</v>
       </c>
-      <c r="D20" s="65"/>
-      <c r="E20" s="64" t="s">
+      <c r="D20" s="64"/>
+      <c r="E20" s="63" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="64" t="s">
+      <c r="A21" s="63" t="s">
         <v>358</v>
       </c>
-      <c r="B21" s="64" t="s">
+      <c r="B21" s="63" t="s">
         <v>306</v>
       </c>
-      <c r="C21" s="64" t="s">
+      <c r="C21" s="63" t="s">
         <v>381</v>
       </c>
-      <c r="D21" s="65"/>
-      <c r="E21" s="64" t="s">
+      <c r="D21" s="64"/>
+      <c r="E21" s="63" t="s">
         <v>142</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added drawings for ALPACA and Optics Lab
</commit_message>
<xml_diff>
--- a/Antonio-Feed/__FeedPartsInventory.xlsx
+++ b/Antonio-Feed/__FeedPartsInventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pollak/Documents/GitHub/Front-Page/Antonio-Feed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FBBDE6F-6D51-AB40-8D23-E28C724EAF1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{510F6DBD-23CF-494F-A1A7-43D649DD396E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-100000" yWindow="600" windowWidth="34200" windowHeight="19940" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-100000" yWindow="600" windowWidth="34200" windowHeight="19940" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts At ATA" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="452">
   <si>
     <t>Antenna Inventory</t>
   </si>
@@ -1396,6 +1396,9 @@
   </si>
   <si>
     <t>5C4-044</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -2195,6 +2198,32 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2206,16 +2235,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2234,22 +2253,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2488,25 +2491,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
-      <c r="D1" s="109"/>
-      <c r="E1" s="109"/>
-      <c r="F1" s="109"/>
-      <c r="G1" s="109"/>
-      <c r="H1" s="110"/>
-      <c r="I1" s="111"/>
-      <c r="J1" s="111"/>
-      <c r="K1" s="110"/>
-      <c r="L1" s="111"/>
-      <c r="M1" s="111"/>
-      <c r="N1" s="111"/>
-      <c r="O1" s="111"/>
-      <c r="P1" s="111"/>
-      <c r="Q1" s="111"/>
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
+      <c r="D1" s="121"/>
+      <c r="E1" s="121"/>
+      <c r="F1" s="121"/>
+      <c r="G1" s="121"/>
+      <c r="H1" s="122"/>
+      <c r="I1" s="123"/>
+      <c r="J1" s="123"/>
+      <c r="K1" s="122"/>
+      <c r="L1" s="123"/>
+      <c r="M1" s="123"/>
+      <c r="N1" s="123"/>
+      <c r="O1" s="123"/>
+      <c r="P1" s="123"/>
+      <c r="Q1" s="123"/>
     </row>
     <row r="2" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -3818,28 +3821,28 @@
       <c r="A58" s="3"/>
     </row>
     <row r="59" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="112"/>
-      <c r="B59" s="107"/>
-      <c r="C59" s="107"/>
+      <c r="A59" s="124"/>
+      <c r="B59" s="119"/>
+      <c r="C59" s="119"/>
     </row>
     <row r="60" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="7"/>
     </row>
     <row r="61" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="106"/>
-      <c r="B61" s="107"/>
-      <c r="C61" s="106"/>
-      <c r="D61" s="107"/>
-      <c r="E61" s="107"/>
-      <c r="F61" s="107"/>
+      <c r="A61" s="118"/>
+      <c r="B61" s="119"/>
+      <c r="C61" s="118"/>
+      <c r="D61" s="119"/>
+      <c r="E61" s="119"/>
+      <c r="F61" s="119"/>
     </row>
     <row r="62" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="106"/>
-      <c r="B62" s="107"/>
-      <c r="C62" s="106"/>
-      <c r="D62" s="107"/>
-      <c r="E62" s="107"/>
-      <c r="F62" s="107"/>
+      <c r="A62" s="118"/>
+      <c r="B62" s="119"/>
+      <c r="C62" s="118"/>
+      <c r="D62" s="119"/>
+      <c r="E62" s="119"/>
+      <c r="F62" s="119"/>
     </row>
     <row r="63" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="64" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4816,20 +4819,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="114" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="115" t="s">
+      <c r="B1" s="115"/>
+      <c r="C1" s="116" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
       <c r="K1" s="9"/>
       <c r="L1" s="9"/>
     </row>
@@ -5305,8 +5308,8 @@
         <f>HYPERLINK("https://drive.google.com/drive/folders/1MyuBrs08Ryi2pvVUeI0hW4p24qsMsUL4","5C4-012")</f>
         <v>5C4-012</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>130</v>
+      <c r="B14" s="103" t="s">
+        <v>126</v>
       </c>
       <c r="C14" s="17" t="s">
         <v>25</v>
@@ -5853,370 +5856,370 @@
       <c r="A28" s="16" t="s">
         <v>407</v>
       </c>
-      <c r="B28" s="124" t="s">
+      <c r="B28" s="107" t="s">
         <v>417</v>
       </c>
-      <c r="C28" s="125"/>
-      <c r="D28" s="126" t="s">
-        <v>25</v>
-      </c>
-      <c r="E28" s="126" t="s">
-        <v>25</v>
-      </c>
-      <c r="F28" s="126" t="s">
-        <v>25</v>
-      </c>
-      <c r="G28" s="127"/>
-      <c r="H28" s="126" t="s">
-        <v>25</v>
-      </c>
-      <c r="I28" s="127"/>
-      <c r="J28" s="127"/>
-      <c r="K28" s="127"/>
-      <c r="L28" s="127"/>
-      <c r="M28" s="128"/>
+      <c r="C28" s="108"/>
+      <c r="D28" s="109" t="s">
+        <v>25</v>
+      </c>
+      <c r="E28" s="109" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28" s="109" t="s">
+        <v>25</v>
+      </c>
+      <c r="G28" s="110"/>
+      <c r="H28" s="109" t="s">
+        <v>25</v>
+      </c>
+      <c r="I28" s="110"/>
+      <c r="J28" s="110"/>
+      <c r="K28" s="110"/>
+      <c r="L28" s="110"/>
+      <c r="M28" s="111"/>
     </row>
     <row r="29" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="123" t="s">
+      <c r="A29" s="106" t="s">
         <v>433</v>
       </c>
-      <c r="B29" s="130" t="s">
+      <c r="B29" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C29" s="54"/>
-      <c r="D29" s="129"/>
-      <c r="E29" s="129"/>
-      <c r="F29" s="129"/>
-      <c r="G29" s="129"/>
-      <c r="H29" s="129"/>
-      <c r="I29" s="129"/>
-      <c r="J29" s="129"/>
-      <c r="K29" s="129"/>
-      <c r="L29" s="129"/>
-      <c r="M29" s="129"/>
+      <c r="D29" s="112"/>
+      <c r="E29" s="112"/>
+      <c r="F29" s="112"/>
+      <c r="G29" s="112"/>
+      <c r="H29" s="112"/>
+      <c r="I29" s="112"/>
+      <c r="J29" s="112"/>
+      <c r="K29" s="112"/>
+      <c r="L29" s="112"/>
+      <c r="M29" s="112"/>
     </row>
     <row r="30" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="123" t="s">
+      <c r="A30" s="106" t="s">
         <v>434</v>
       </c>
-      <c r="B30" s="130" t="s">
+      <c r="B30" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C30" s="54"/>
-      <c r="D30" s="129"/>
-      <c r="E30" s="129"/>
-      <c r="F30" s="129"/>
-      <c r="G30" s="129"/>
-      <c r="H30" s="129"/>
-      <c r="I30" s="129"/>
-      <c r="J30" s="129"/>
-      <c r="K30" s="129"/>
-      <c r="L30" s="129"/>
-      <c r="M30" s="129"/>
+      <c r="D30" s="112"/>
+      <c r="E30" s="112"/>
+      <c r="F30" s="112"/>
+      <c r="G30" s="112"/>
+      <c r="H30" s="112"/>
+      <c r="I30" s="112"/>
+      <c r="J30" s="112"/>
+      <c r="K30" s="112"/>
+      <c r="L30" s="112"/>
+      <c r="M30" s="112"/>
     </row>
     <row r="31" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="123" t="s">
+      <c r="A31" s="106" t="s">
         <v>435</v>
       </c>
-      <c r="B31" s="130" t="s">
+      <c r="B31" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C31" s="54"/>
-      <c r="D31" s="129"/>
-      <c r="E31" s="129"/>
-      <c r="F31" s="129"/>
-      <c r="G31" s="129"/>
-      <c r="H31" s="129"/>
-      <c r="I31" s="129"/>
-      <c r="J31" s="129"/>
-      <c r="K31" s="129"/>
-      <c r="L31" s="129"/>
-      <c r="M31" s="129"/>
+      <c r="D31" s="112"/>
+      <c r="E31" s="112"/>
+      <c r="F31" s="112"/>
+      <c r="G31" s="112"/>
+      <c r="H31" s="112"/>
+      <c r="I31" s="112"/>
+      <c r="J31" s="112"/>
+      <c r="K31" s="112"/>
+      <c r="L31" s="112"/>
+      <c r="M31" s="112"/>
     </row>
     <row r="32" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="123" t="s">
+      <c r="A32" s="106" t="s">
         <v>436</v>
       </c>
-      <c r="B32" s="130" t="s">
+      <c r="B32" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C32" s="54"/>
-      <c r="D32" s="129"/>
-      <c r="E32" s="129"/>
-      <c r="F32" s="129"/>
-      <c r="G32" s="129"/>
-      <c r="H32" s="129"/>
-      <c r="I32" s="129"/>
-      <c r="J32" s="129"/>
-      <c r="K32" s="129"/>
-      <c r="L32" s="129"/>
-      <c r="M32" s="129"/>
+      <c r="D32" s="112"/>
+      <c r="E32" s="112"/>
+      <c r="F32" s="112"/>
+      <c r="G32" s="112"/>
+      <c r="H32" s="112"/>
+      <c r="I32" s="112"/>
+      <c r="J32" s="112"/>
+      <c r="K32" s="112"/>
+      <c r="L32" s="112"/>
+      <c r="M32" s="112"/>
     </row>
     <row r="33" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="123" t="s">
+      <c r="A33" s="106" t="s">
         <v>437</v>
       </c>
-      <c r="B33" s="130" t="s">
+      <c r="B33" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C33" s="54"/>
-      <c r="D33" s="129"/>
-      <c r="E33" s="129"/>
-      <c r="F33" s="129"/>
-      <c r="G33" s="129"/>
-      <c r="H33" s="129"/>
-      <c r="I33" s="129"/>
-      <c r="J33" s="129"/>
-      <c r="K33" s="129"/>
-      <c r="L33" s="129"/>
-      <c r="M33" s="129"/>
+      <c r="D33" s="112"/>
+      <c r="E33" s="112"/>
+      <c r="F33" s="112"/>
+      <c r="G33" s="112"/>
+      <c r="H33" s="112"/>
+      <c r="I33" s="112"/>
+      <c r="J33" s="112"/>
+      <c r="K33" s="112"/>
+      <c r="L33" s="112"/>
+      <c r="M33" s="112"/>
     </row>
     <row r="34" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="123" t="s">
+      <c r="A34" s="106" t="s">
         <v>438</v>
       </c>
-      <c r="B34" s="130" t="s">
+      <c r="B34" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C34" s="54"/>
-      <c r="D34" s="129"/>
-      <c r="E34" s="129"/>
-      <c r="F34" s="129"/>
-      <c r="G34" s="129"/>
-      <c r="H34" s="129"/>
-      <c r="I34" s="129"/>
-      <c r="J34" s="129"/>
-      <c r="K34" s="129"/>
-      <c r="L34" s="129"/>
-      <c r="M34" s="129"/>
+      <c r="D34" s="112"/>
+      <c r="E34" s="112"/>
+      <c r="F34" s="112"/>
+      <c r="G34" s="112"/>
+      <c r="H34" s="112"/>
+      <c r="I34" s="112"/>
+      <c r="J34" s="112"/>
+      <c r="K34" s="112"/>
+      <c r="L34" s="112"/>
+      <c r="M34" s="112"/>
     </row>
     <row r="35" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="123" t="s">
+      <c r="A35" s="106" t="s">
         <v>439</v>
       </c>
-      <c r="B35" s="130" t="s">
+      <c r="B35" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C35" s="54"/>
-      <c r="D35" s="129"/>
-      <c r="E35" s="129"/>
-      <c r="F35" s="129"/>
-      <c r="G35" s="129"/>
-      <c r="H35" s="129"/>
-      <c r="I35" s="129"/>
-      <c r="J35" s="129"/>
-      <c r="K35" s="129"/>
-      <c r="L35" s="129"/>
-      <c r="M35" s="129"/>
+      <c r="D35" s="112"/>
+      <c r="E35" s="112"/>
+      <c r="F35" s="112"/>
+      <c r="G35" s="112"/>
+      <c r="H35" s="112"/>
+      <c r="I35" s="112"/>
+      <c r="J35" s="112"/>
+      <c r="K35" s="112"/>
+      <c r="L35" s="112"/>
+      <c r="M35" s="112"/>
     </row>
     <row r="36" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="123" t="s">
+      <c r="A36" s="106" t="s">
         <v>440</v>
       </c>
-      <c r="B36" s="130" t="s">
+      <c r="B36" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C36" s="54"/>
-      <c r="D36" s="129"/>
-      <c r="E36" s="129"/>
-      <c r="F36" s="129"/>
-      <c r="G36" s="129"/>
-      <c r="H36" s="129"/>
-      <c r="I36" s="129"/>
-      <c r="J36" s="129"/>
-      <c r="K36" s="129"/>
-      <c r="L36" s="129"/>
-      <c r="M36" s="129"/>
+      <c r="D36" s="112"/>
+      <c r="E36" s="112"/>
+      <c r="F36" s="112"/>
+      <c r="G36" s="112"/>
+      <c r="H36" s="112"/>
+      <c r="I36" s="112"/>
+      <c r="J36" s="112"/>
+      <c r="K36" s="112"/>
+      <c r="L36" s="112"/>
+      <c r="M36" s="112"/>
     </row>
     <row r="37" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="123" t="s">
+      <c r="A37" s="106" t="s">
         <v>441</v>
       </c>
-      <c r="B37" s="130" t="s">
+      <c r="B37" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C37" s="54"/>
-      <c r="D37" s="129"/>
-      <c r="E37" s="129"/>
-      <c r="F37" s="129"/>
-      <c r="G37" s="129"/>
-      <c r="H37" s="129"/>
-      <c r="I37" s="129"/>
-      <c r="J37" s="129"/>
-      <c r="K37" s="129"/>
-      <c r="L37" s="129"/>
-      <c r="M37" s="129"/>
+      <c r="D37" s="112"/>
+      <c r="E37" s="112"/>
+      <c r="F37" s="112"/>
+      <c r="G37" s="112"/>
+      <c r="H37" s="112"/>
+      <c r="I37" s="112"/>
+      <c r="J37" s="112"/>
+      <c r="K37" s="112"/>
+      <c r="L37" s="112"/>
+      <c r="M37" s="112"/>
     </row>
     <row r="38" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="123" t="s">
+      <c r="A38" s="106" t="s">
         <v>442</v>
       </c>
-      <c r="B38" s="130" t="s">
+      <c r="B38" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C38" s="54"/>
-      <c r="D38" s="129"/>
-      <c r="E38" s="129"/>
-      <c r="F38" s="129"/>
-      <c r="G38" s="129"/>
-      <c r="H38" s="129"/>
-      <c r="I38" s="129"/>
-      <c r="J38" s="129"/>
-      <c r="K38" s="129"/>
-      <c r="L38" s="129"/>
-      <c r="M38" s="129"/>
+      <c r="D38" s="112"/>
+      <c r="E38" s="112"/>
+      <c r="F38" s="112"/>
+      <c r="G38" s="112"/>
+      <c r="H38" s="112"/>
+      <c r="I38" s="112"/>
+      <c r="J38" s="112"/>
+      <c r="K38" s="112"/>
+      <c r="L38" s="112"/>
+      <c r="M38" s="112"/>
     </row>
     <row r="39" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="123" t="s">
+      <c r="A39" s="106" t="s">
         <v>443</v>
       </c>
-      <c r="B39" s="130" t="s">
+      <c r="B39" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C39" s="54"/>
-      <c r="D39" s="129"/>
-      <c r="E39" s="129"/>
-      <c r="F39" s="129"/>
-      <c r="G39" s="129"/>
-      <c r="H39" s="129"/>
-      <c r="I39" s="129"/>
-      <c r="J39" s="129"/>
-      <c r="K39" s="129"/>
-      <c r="L39" s="129"/>
-      <c r="M39" s="129"/>
+      <c r="D39" s="112"/>
+      <c r="E39" s="112"/>
+      <c r="F39" s="112"/>
+      <c r="G39" s="112"/>
+      <c r="H39" s="112"/>
+      <c r="I39" s="112"/>
+      <c r="J39" s="112"/>
+      <c r="K39" s="112"/>
+      <c r="L39" s="112"/>
+      <c r="M39" s="112"/>
     </row>
     <row r="40" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="123" t="s">
+      <c r="A40" s="106" t="s">
         <v>444</v>
       </c>
-      <c r="B40" s="130" t="s">
+      <c r="B40" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C40" s="54"/>
-      <c r="D40" s="129"/>
-      <c r="E40" s="129"/>
-      <c r="F40" s="129"/>
-      <c r="G40" s="129"/>
-      <c r="H40" s="129"/>
-      <c r="I40" s="129"/>
-      <c r="J40" s="129"/>
-      <c r="K40" s="129"/>
-      <c r="L40" s="129"/>
-      <c r="M40" s="129"/>
+      <c r="D40" s="112"/>
+      <c r="E40" s="112"/>
+      <c r="F40" s="112"/>
+      <c r="G40" s="112"/>
+      <c r="H40" s="112"/>
+      <c r="I40" s="112"/>
+      <c r="J40" s="112"/>
+      <c r="K40" s="112"/>
+      <c r="L40" s="112"/>
+      <c r="M40" s="112"/>
     </row>
     <row r="41" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="123" t="s">
+      <c r="A41" s="106" t="s">
         <v>445</v>
       </c>
-      <c r="B41" s="130" t="s">
+      <c r="B41" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C41" s="54"/>
-      <c r="D41" s="129"/>
-      <c r="E41" s="129"/>
-      <c r="F41" s="129"/>
-      <c r="G41" s="129"/>
-      <c r="H41" s="129"/>
-      <c r="I41" s="129"/>
-      <c r="J41" s="129"/>
-      <c r="K41" s="129"/>
-      <c r="L41" s="129"/>
-      <c r="M41" s="129"/>
+      <c r="D41" s="112"/>
+      <c r="E41" s="112"/>
+      <c r="F41" s="112"/>
+      <c r="G41" s="112"/>
+      <c r="H41" s="112"/>
+      <c r="I41" s="112"/>
+      <c r="J41" s="112"/>
+      <c r="K41" s="112"/>
+      <c r="L41" s="112"/>
+      <c r="M41" s="112"/>
     </row>
     <row r="42" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="123" t="s">
+      <c r="A42" s="106" t="s">
         <v>446</v>
       </c>
-      <c r="B42" s="130" t="s">
+      <c r="B42" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C42" s="54"/>
-      <c r="D42" s="129"/>
-      <c r="E42" s="129"/>
-      <c r="F42" s="129"/>
-      <c r="G42" s="129"/>
-      <c r="H42" s="129"/>
-      <c r="I42" s="129"/>
-      <c r="J42" s="129"/>
-      <c r="K42" s="129"/>
-      <c r="L42" s="129"/>
-      <c r="M42" s="129"/>
+      <c r="D42" s="112"/>
+      <c r="E42" s="112"/>
+      <c r="F42" s="112"/>
+      <c r="G42" s="112"/>
+      <c r="H42" s="112"/>
+      <c r="I42" s="112"/>
+      <c r="J42" s="112"/>
+      <c r="K42" s="112"/>
+      <c r="L42" s="112"/>
+      <c r="M42" s="112"/>
     </row>
     <row r="43" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="123" t="s">
+      <c r="A43" s="106" t="s">
         <v>447</v>
       </c>
-      <c r="B43" s="130" t="s">
+      <c r="B43" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C43" s="54"/>
-      <c r="D43" s="129"/>
-      <c r="E43" s="129"/>
-      <c r="F43" s="129"/>
-      <c r="G43" s="129"/>
-      <c r="H43" s="129"/>
-      <c r="I43" s="129"/>
-      <c r="J43" s="129"/>
-      <c r="K43" s="129"/>
-      <c r="L43" s="129"/>
-      <c r="M43" s="129"/>
+      <c r="D43" s="112"/>
+      <c r="E43" s="112"/>
+      <c r="F43" s="112"/>
+      <c r="G43" s="112"/>
+      <c r="H43" s="112"/>
+      <c r="I43" s="112"/>
+      <c r="J43" s="112"/>
+      <c r="K43" s="112"/>
+      <c r="L43" s="112"/>
+      <c r="M43" s="112"/>
     </row>
     <row r="44" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="123" t="s">
+      <c r="A44" s="106" t="s">
         <v>448</v>
       </c>
-      <c r="B44" s="130" t="s">
+      <c r="B44" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C44" s="54"/>
-      <c r="D44" s="129"/>
-      <c r="E44" s="129"/>
-      <c r="F44" s="129"/>
-      <c r="G44" s="129"/>
-      <c r="H44" s="129"/>
-      <c r="I44" s="129"/>
-      <c r="J44" s="129"/>
-      <c r="K44" s="129"/>
-      <c r="L44" s="129"/>
-      <c r="M44" s="129"/>
+      <c r="D44" s="112"/>
+      <c r="E44" s="112"/>
+      <c r="F44" s="112"/>
+      <c r="G44" s="112"/>
+      <c r="H44" s="112"/>
+      <c r="I44" s="112"/>
+      <c r="J44" s="112"/>
+      <c r="K44" s="112"/>
+      <c r="L44" s="112"/>
+      <c r="M44" s="112"/>
     </row>
     <row r="45" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="123" t="s">
+      <c r="A45" s="106" t="s">
         <v>449</v>
       </c>
-      <c r="B45" s="130" t="s">
+      <c r="B45" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C45" s="54"/>
-      <c r="D45" s="129"/>
-      <c r="E45" s="129"/>
-      <c r="F45" s="129"/>
-      <c r="G45" s="129"/>
-      <c r="H45" s="129"/>
-      <c r="I45" s="129"/>
-      <c r="J45" s="129"/>
-      <c r="K45" s="129"/>
-      <c r="L45" s="129"/>
-      <c r="M45" s="129"/>
+      <c r="D45" s="112"/>
+      <c r="E45" s="112"/>
+      <c r="F45" s="112"/>
+      <c r="G45" s="112"/>
+      <c r="H45" s="112"/>
+      <c r="I45" s="112"/>
+      <c r="J45" s="112"/>
+      <c r="K45" s="112"/>
+      <c r="L45" s="112"/>
+      <c r="M45" s="112"/>
     </row>
     <row r="46" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="123" t="s">
+      <c r="A46" s="106" t="s">
         <v>450</v>
       </c>
-      <c r="B46" s="130" t="s">
+      <c r="B46" s="113" t="s">
         <v>385</v>
       </c>
       <c r="C46" s="54"/>
-      <c r="D46" s="129"/>
-      <c r="E46" s="129"/>
-      <c r="F46" s="129"/>
-      <c r="G46" s="129"/>
-      <c r="H46" s="129"/>
-      <c r="I46" s="129"/>
-      <c r="J46" s="129"/>
-      <c r="K46" s="129"/>
-      <c r="L46" s="129"/>
-      <c r="M46" s="129"/>
+      <c r="D46" s="112"/>
+      <c r="E46" s="112"/>
+      <c r="F46" s="112"/>
+      <c r="G46" s="112"/>
+      <c r="H46" s="112"/>
+      <c r="I46" s="112"/>
+      <c r="J46" s="112"/>
+      <c r="K46" s="112"/>
+      <c r="L46" s="112"/>
+      <c r="M46" s="112"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6239,14 +6242,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="115" t="s">
+      <c r="A1" s="116" t="s">
         <v>330</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
       <c r="G1" s="61"/>
       <c r="H1" s="61"/>
       <c r="I1" s="61"/>
@@ -6555,7 +6558,7 @@
         <v>360</v>
       </c>
       <c r="F14" s="62" t="s">
-        <v>42</v>
+        <v>451</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -6921,20 +6924,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="125" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="118"/>
-      <c r="C1" s="117" t="s">
+      <c r="B1" s="126"/>
+      <c r="C1" s="125" t="s">
         <v>251</v>
       </c>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="118"/>
+      <c r="D1" s="127"/>
+      <c r="E1" s="127"/>
+      <c r="F1" s="127"/>
+      <c r="G1" s="127"/>
+      <c r="H1" s="127"/>
+      <c r="I1" s="127"/>
+      <c r="J1" s="126"/>
     </row>
     <row r="2" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="37" t="s">
@@ -7492,21 +7495,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="120" t="s">
+      <c r="A1" s="128" t="s">
         <v>297</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
+      <c r="B1" s="129"/>
+      <c r="C1" s="129"/>
       <c r="D1" s="81"/>
-      <c r="E1" s="110" t="s">
+      <c r="E1" s="122" t="s">
         <v>397</v>
       </c>
-      <c r="F1" s="110"/>
-      <c r="G1" s="110"/>
-      <c r="H1" s="122" t="s">
+      <c r="F1" s="122"/>
+      <c r="G1" s="122"/>
+      <c r="H1" s="130" t="s">
         <v>410</v>
       </c>
-      <c r="I1" s="122"/>
+      <c r="I1" s="130"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="82" t="s">

</xml_diff>